<commit_message>
Rajasthan automation  Vendor id is working
</commit_message>
<xml_diff>
--- a/RAJ_MINING_DEVICES.xlsx
+++ b/RAJ_MINING_DEVICES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Playwright Leaning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EFAAB8D-DE2C-4CBB-9A68-9DB2A9D57B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC512F00-8FFC-4112-A7FC-CA2EAF144BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7474299F-CE95-4174-832F-DFBC93F2AF1D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
     <t>Result</t>
   </si>
   <si>
-    <t>RJ19GK8694</t>
+    <t>RJ20GD1368</t>
   </si>
 </sst>
 </file>
@@ -423,32 +423,32 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>865510084807736</v>
+      <c r="A2" s="1">
+        <v>865510084659640</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>865510084807736</v>
+      <c r="A3" s="1">
+        <v>865510084659640</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>865510084807736</v>
+      <c r="A4" s="1">
+        <v>865510084659640</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>865510084807736</v>
+      <c r="A5" s="1">
+        <v>865510084659640</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
now it will ignore used range , checking vendor id and test id is also skipped
</commit_message>
<xml_diff>
--- a/RAJ_MINING_DEVICES.xlsx
+++ b/RAJ_MINING_DEVICES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Playwright Leaning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC512F00-8FFC-4112-A7FC-CA2EAF144BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148B980F-C8F2-4595-B055-2A28DC172851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7474299F-CE95-4174-832F-DFBC93F2AF1D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>IMEI</t>
   </si>
@@ -431,28 +431,16 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="1">
-        <v>865510084659640</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>3</v>
-      </c>
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="1">
-        <v>865510084659640</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>3</v>
-      </c>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="1">
-        <v>865510084659640</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>3</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
actually now all input steps are removed it wil not wait after confirming imei and Vehicle number
</commit_message>
<xml_diff>
--- a/RAJ_MINING_DEVICES.xlsx
+++ b/RAJ_MINING_DEVICES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Playwright Leaning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148B980F-C8F2-4595-B055-2A28DC172851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DDE5B63-1D0C-49BA-AEF9-5E03E1B884BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7474299F-CE95-4174-832F-DFBC93F2AF1D}"/>
   </bookViews>
@@ -45,7 +45,7 @@
     <t>Result</t>
   </si>
   <si>
-    <t>RJ20GD1368</t>
+    <t>HR849555</t>
   </si>
 </sst>
 </file>
@@ -424,7 +424,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
-        <v>865510084659640</v>
+        <v>869645080504394</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
empty cell will not take none value now its working properly
</commit_message>
<xml_diff>
--- a/RAJ_MINING_DEVICES.xlsx
+++ b/RAJ_MINING_DEVICES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Playwright Leaning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DDE5B63-1D0C-49BA-AEF9-5E03E1B884BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A2C05E6-6DBF-4ACC-BEE4-F022C4F6B8C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7474299F-CE95-4174-832F-DFBC93F2AF1D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="4">
   <si>
     <t>IMEI</t>
   </si>
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C8B192C-6556-4B92-A17D-B5AFAC06BD13}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.81640625" bestFit="1" customWidth="1"/>
@@ -431,18 +431,47 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
+      <c r="A3" s="1">
+        <v>869645080504394</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
+      <c r="A4" s="1">
+        <v>869645080504394</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
+      <c r="A5" s="1">
+        <v>869645080504394</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="1">
+        <v>869645080504394</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="1">
+        <v>869645080504394</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
default file is changed now txt file path is not needed
</commit_message>
<xml_diff>
--- a/RAJ_MINING_DEVICES.xlsx
+++ b/RAJ_MINING_DEVICES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Playwright Leaning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A2C05E6-6DBF-4ACC-BEE4-F022C4F6B8C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E652AAFA-D5D3-4417-A99A-9FB930D352E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7474299F-CE95-4174-832F-DFBC93F2AF1D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="5">
   <si>
     <t>IMEI</t>
   </si>
@@ -46,6 +46,9 @@
   </si>
   <si>
     <t>HR849555</t>
+  </si>
+  <si>
+    <t>RJ52GB3798</t>
   </si>
 </sst>
 </file>
@@ -424,26 +427,26 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
-        <v>869645080504394</v>
+        <v>862491079224794</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
-        <v>869645080504394</v>
+        <v>862491079224794</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
-        <v>869645080504394</v>
+        <v>862491079224794</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
login  function is changed
</commit_message>
<xml_diff>
--- a/RAJ_MINING_DEVICES.xlsx
+++ b/RAJ_MINING_DEVICES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Playwright Leaning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E652AAFA-D5D3-4417-A99A-9FB930D352E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86AC34CB-F055-4B42-8E8C-44540F71E1DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7474299F-CE95-4174-832F-DFBC93F2AF1D}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>IMEI</t>
   </si>
@@ -45,17 +46,14 @@
     <t>Result</t>
   </si>
   <si>
-    <t>HR849555</t>
-  </si>
-  <si>
-    <t>RJ52GB3798</t>
+    <t>BR03GC2329</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -66,6 +64,12 @@
     <font>
       <sz val="7"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -90,9 +94,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -411,7 +416,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -426,52 +431,32 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="1">
-        <v>862491079224794</v>
+      <c r="A2" s="2">
+        <v>862491072743709</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="1">
-        <v>862491079224794</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="1">
-        <v>862491079224794</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="1">
-        <v>869645080504394</v>
-      </c>
-      <c r="B5" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+    </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="1">
-        <v>869645080504394</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>3</v>
-      </c>
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="1">
-        <v>869645080504394</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>3</v>
-      </c>
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>